<commit_message>
added 3.3v regulator according to schematic
</commit_message>
<xml_diff>
--- a/PCB/BOM.xlsx
+++ b/PCB/BOM.xlsx
@@ -4,14 +4,14 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="BOM_Board1_PCB_2026-04-10" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="BOM_Board1_PCB2_2026-04-13" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="191">
   <si>
     <t>No.</t>
   </si>
@@ -73,7 +73,7 @@
     <t>100nF</t>
   </si>
   <si>
-    <t>C8,C9,C10,C11,C12,C16</t>
+    <t>C8,C9,C10,C11,C12,C16,C17,C19</t>
   </si>
   <si>
     <t>C0402</t>
@@ -94,7 +94,7 @@
     <t>10uF</t>
   </si>
   <si>
-    <t>C14</t>
+    <t>C14,C18</t>
   </si>
   <si>
     <t>CL10A106MQ8NNNC</t>
@@ -253,7 +253,7 @@
     <t>2.54-1*1P针</t>
   </si>
   <si>
-    <t>p8,zdc</t>
+    <t>p8,p9,zdc</t>
   </si>
   <si>
     <t>HDR-TH_1P-P2.54-V-M</t>
@@ -283,163 +283,166 @@
     <t>14</t>
   </si>
   <si>
+    <t>1kΩ</t>
+  </si>
+  <si>
+    <t>R19,R21,R22</t>
+  </si>
+  <si>
+    <t>R1206</t>
+  </si>
+  <si>
+    <t>1206W4J0102T5E</t>
+  </si>
+  <si>
+    <t>UNI-ROYAL(厚声)</t>
+  </si>
+  <si>
+    <t>C1469</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>1MΩ</t>
+  </si>
+  <si>
+    <t>R20</t>
+  </si>
+  <si>
+    <t>1206W4F1004T5E</t>
+  </si>
+  <si>
+    <t>C17927</t>
+  </si>
+  <si>
+    <t>16</t>
+  </si>
+  <si>
+    <t>10kΩ</t>
+  </si>
+  <si>
+    <t>R23</t>
+  </si>
+  <si>
+    <t>R0805</t>
+  </si>
+  <si>
+    <t>0805W8J0103T5E</t>
+  </si>
+  <si>
+    <t>C25612</t>
+  </si>
+  <si>
+    <t>17</t>
+  </si>
+  <si>
+    <t>190pF@1kHz</t>
+  </si>
+  <si>
+    <t>R24</t>
+  </si>
+  <si>
+    <t>RES-TH_L12.5-W6.7-P7.50-D1.2</t>
+  </si>
+  <si>
+    <t>10D471K</t>
+  </si>
+  <si>
+    <t>RUILON(瑞隆源)</t>
+  </si>
+  <si>
+    <t>C8760</t>
+  </si>
+  <si>
+    <t>18</t>
+  </si>
+  <si>
+    <t>47kΩ</t>
+  </si>
+  <si>
+    <t>R30,R43</t>
+  </si>
+  <si>
+    <t>R1210</t>
+  </si>
+  <si>
+    <t>1210W2F4702T5E</t>
+  </si>
+  <si>
+    <t>C620684</t>
+  </si>
+  <si>
+    <t>19</t>
+  </si>
+  <si>
+    <t>1.4kΩ</t>
+  </si>
+  <si>
+    <t>R31,R32,R33,R34,R35</t>
+  </si>
+  <si>
+    <t>R0402</t>
+  </si>
+  <si>
+    <t>0402WGF1401TCE</t>
+  </si>
+  <si>
+    <t>C39650</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>220Ω</t>
+  </si>
+  <si>
+    <t>R36,R37,R38,R39,R40</t>
+  </si>
+  <si>
+    <t>0805W8F2200T5E</t>
+  </si>
+  <si>
+    <t>C17557</t>
+  </si>
+  <si>
+    <t>21</t>
+  </si>
+  <si>
+    <t>10Ω</t>
+  </si>
+  <si>
+    <t>R42</t>
+  </si>
+  <si>
+    <t>RES-TH_BD5.0-L15.5-P19.50-D0.7</t>
+  </si>
+  <si>
+    <t>KNP03SJ0100A10</t>
+  </si>
+  <si>
+    <t>C74771</t>
+  </si>
+  <si>
+    <t>22</t>
+  </si>
+  <si>
     <t>470Ω</t>
   </si>
   <si>
-    <t>R4,R12,R13,R14,R15</t>
-  </si>
-  <si>
-    <t>R2512</t>
-  </si>
-  <si>
-    <t>25121WJ0471T4E</t>
-  </si>
-  <si>
-    <t>UNI-ROYAL(厚声)</t>
-  </si>
-  <si>
-    <t>C24919</t>
-  </si>
-  <si>
-    <t>15</t>
-  </si>
-  <si>
-    <t>1kΩ</t>
-  </si>
-  <si>
-    <t>R19,R21,R22</t>
-  </si>
-  <si>
-    <t>R1206</t>
-  </si>
-  <si>
-    <t>1206W4J0102T5E</t>
-  </si>
-  <si>
-    <t>C1469</t>
-  </si>
-  <si>
-    <t>16</t>
-  </si>
-  <si>
-    <t>1MΩ</t>
-  </si>
-  <si>
-    <t>R20</t>
-  </si>
-  <si>
-    <t>1206W4F1004T5E</t>
-  </si>
-  <si>
-    <t>C17927</t>
-  </si>
-  <si>
-    <t>17</t>
-  </si>
-  <si>
-    <t>10kΩ</t>
-  </si>
-  <si>
-    <t>R23</t>
-  </si>
-  <si>
-    <t>R0805</t>
-  </si>
-  <si>
-    <t>0805W8J0103T5E</t>
-  </si>
-  <si>
-    <t>C25612</t>
-  </si>
-  <si>
-    <t>18</t>
-  </si>
-  <si>
-    <t>190pF@1kHz</t>
-  </si>
-  <si>
-    <t>R24</t>
-  </si>
-  <si>
-    <t>RES-TH_L12.5-W6.7-P7.50-D1.2</t>
-  </si>
-  <si>
-    <t>10D471K</t>
-  </si>
-  <si>
-    <t>RUILON(瑞隆源)</t>
-  </si>
-  <si>
-    <t>C8760</t>
-  </si>
-  <si>
-    <t>19</t>
-  </si>
-  <si>
-    <t>47kΩ</t>
-  </si>
-  <si>
-    <t>R30,R43</t>
-  </si>
-  <si>
-    <t>R1210</t>
-  </si>
-  <si>
-    <t>1210W2F4702T5E</t>
-  </si>
-  <si>
-    <t>C620684</t>
-  </si>
-  <si>
-    <t>20</t>
-  </si>
-  <si>
-    <t>1.4kΩ</t>
-  </si>
-  <si>
-    <t>R31,R32,R33,R34,R35</t>
-  </si>
-  <si>
-    <t>R0402</t>
-  </si>
-  <si>
-    <t>0402WGF1401TCE</t>
-  </si>
-  <si>
-    <t>C39650</t>
-  </si>
-  <si>
-    <t>21</t>
-  </si>
-  <si>
-    <t>220Ω</t>
-  </si>
-  <si>
-    <t>R36,R37,R38,R39,R40</t>
-  </si>
-  <si>
-    <t>0805W8F2200T5E</t>
-  </si>
-  <si>
-    <t>C17557</t>
-  </si>
-  <si>
-    <t>22</t>
-  </si>
-  <si>
-    <t>10Ω</t>
-  </si>
-  <si>
-    <t>R42</t>
-  </si>
-  <si>
-    <t>RES-TH_BD5.0-L15.5-P19.50-D0.7</t>
-  </si>
-  <si>
-    <t>KNP03SJ0100A10</t>
-  </si>
-  <si>
-    <t>C74771</t>
+    <t>R44,R45,R46,R47,R48</t>
+  </si>
+  <si>
+    <t>R0207</t>
+  </si>
+  <si>
+    <t>MMB02070C4700FB200</t>
+  </si>
+  <si>
+    <t>VISHAY(威世)</t>
+  </si>
+  <si>
+    <t>C2075148</t>
   </si>
   <si>
     <t>23</t>
@@ -514,7 +517,7 @@
     <t>DS1021-1x2SF11-B</t>
   </si>
   <si>
-    <t>U14,U15,U16</t>
+    <t>U14,U15,U16,U23</t>
   </si>
   <si>
     <t>HDR-TH_2P-P2.54-V-M</t>
@@ -535,7 +538,7 @@
     <t>U17,U18,U19,U20,U21</t>
   </si>
   <si>
-    <t>SMD-6_L8.8-W6.4-P2.54-LS9.4-BL</t>
+    <t>MOC3053_NoPin5</t>
   </si>
   <si>
     <t>onsemi(安森美)</t>
@@ -545,6 +548,24 @@
   </si>
   <si>
     <t>29</t>
+  </si>
+  <si>
+    <t>AMS1117-3.3V</t>
+  </si>
+  <si>
+    <t>U22</t>
+  </si>
+  <si>
+    <t>SOT-223-4_L6.5-W3.5-P2.30-LS7.0-BR</t>
+  </si>
+  <si>
+    <t>WPMtek(维攀)</t>
+  </si>
+  <si>
+    <t>C2688239</t>
+  </si>
+  <si>
+    <t>30</t>
   </si>
   <si>
     <t>8MHz</t>
@@ -939,7 +960,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J31"/>
+  <dimension ref="A1:J32"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="10" width="20" customWidth="1"/>
@@ -1014,7 +1035,7 @@
         <v>18</v>
       </c>
       <c r="B3">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C3" t="s">
         <v>19</v>
@@ -1046,7 +1067,7 @@
         <v>25</v>
       </c>
       <c r="B4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C4" t="s">
         <v>26</v>
@@ -1334,7 +1355,7 @@
         <v>78</v>
       </c>
       <c r="B13">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C13" t="s">
         <v>79</v>
@@ -1398,7 +1419,7 @@
         <v>89</v>
       </c>
       <c r="B15">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C15" t="s">
         <v>90</v>
@@ -1430,7 +1451,7 @@
         <v>96</v>
       </c>
       <c r="B16">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C16" t="s">
         <v>97</v>
@@ -1439,19 +1460,19 @@
         <v>98</v>
       </c>
       <c r="E16" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="F16" t="s">
         <v>97</v>
       </c>
       <c r="G16" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H16" t="s">
         <v>94</v>
       </c>
       <c r="I16" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="J16" t="s">
         <v>17</v>
@@ -1459,22 +1480,22 @@
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B17">
         <v>1</v>
       </c>
       <c r="C17" t="s">
+        <v>102</v>
+      </c>
+      <c r="D17" t="s">
         <v>103</v>
       </c>
-      <c r="D17" t="s">
+      <c r="E17" t="s">
         <v>104</v>
       </c>
-      <c r="E17" t="s">
-        <v>99</v>
-      </c>
       <c r="F17" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="G17" t="s">
         <v>105</v>
@@ -1512,10 +1533,10 @@
         <v>111</v>
       </c>
       <c r="H18" t="s">
-        <v>94</v>
+        <v>112</v>
       </c>
       <c r="I18" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J18" t="s">
         <v>17</v>
@@ -1523,28 +1544,28 @@
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B19">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C19" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D19" t="s">
+        <v>116</v>
+      </c>
+      <c r="E19" t="s">
+        <v>117</v>
+      </c>
+      <c r="F19" t="s">
         <v>115</v>
       </c>
-      <c r="E19" t="s">
-        <v>116</v>
-      </c>
-      <c r="F19" t="s">
-        <v>114</v>
-      </c>
       <c r="G19" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="H19" t="s">
-        <v>118</v>
+        <v>94</v>
       </c>
       <c r="I19" t="s">
         <v>119</v>
@@ -1558,7 +1579,7 @@
         <v>120</v>
       </c>
       <c r="B20">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C20" t="s">
         <v>121</v>
@@ -1599,19 +1620,19 @@
         <v>128</v>
       </c>
       <c r="E21" t="s">
-        <v>129</v>
+        <v>104</v>
       </c>
       <c r="F21" t="s">
         <v>127</v>
       </c>
       <c r="G21" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H21" t="s">
         <v>94</v>
       </c>
       <c r="I21" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="J21" t="s">
         <v>17</v>
@@ -1619,22 +1640,22 @@
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>131</v>
+      </c>
+      <c r="B22">
+        <v>1</v>
+      </c>
+      <c r="C22" t="s">
         <v>132</v>
       </c>
-      <c r="B22">
-        <v>5</v>
-      </c>
-      <c r="C22" t="s">
+      <c r="D22" t="s">
         <v>133</v>
       </c>
-      <c r="D22" t="s">
+      <c r="E22" t="s">
         <v>134</v>
       </c>
-      <c r="E22" t="s">
-        <v>110</v>
-      </c>
       <c r="F22" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G22" t="s">
         <v>135</v>
@@ -1654,7 +1675,7 @@
         <v>137</v>
       </c>
       <c r="B23">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C23" t="s">
         <v>138</v>
@@ -1672,10 +1693,10 @@
         <v>141</v>
       </c>
       <c r="H23" t="s">
-        <v>94</v>
+        <v>142</v>
       </c>
       <c r="I23" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="J23" t="s">
         <v>17</v>
@@ -1683,31 +1704,31 @@
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B24">
         <v>1</v>
       </c>
       <c r="C24" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D24" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E24" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F24" t="s">
         <v>41</v>
       </c>
       <c r="G24" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="H24" t="s">
         <v>54</v>
       </c>
       <c r="I24" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="J24" t="s">
         <v>17</v>
@@ -1715,31 +1736,31 @@
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B25">
         <v>1</v>
       </c>
       <c r="C25" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D25" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="E25" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F25" t="s">
         <v>41</v>
       </c>
       <c r="G25" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="H25" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="I25" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J25" t="s">
         <v>17</v>
@@ -1747,31 +1768,31 @@
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B26">
         <v>1</v>
       </c>
       <c r="C26" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D26" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E26" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F26" t="s">
         <v>41</v>
       </c>
       <c r="G26" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H26" t="s">
         <v>87</v>
       </c>
       <c r="I26" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J26" t="s">
         <v>17</v>
@@ -1779,31 +1800,31 @@
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B27">
         <v>1</v>
       </c>
       <c r="C27" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D27" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="E27" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F27" t="s">
         <v>41</v>
       </c>
       <c r="G27" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H27" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="I27" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J27" t="s">
         <v>17</v>
@@ -1811,31 +1832,31 @@
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B28">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C28" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D28" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="E28" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="F28" t="s">
         <v>41</v>
       </c>
       <c r="G28" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="H28" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="I28" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="J28" t="s">
         <v>17</v>
@@ -1843,31 +1864,31 @@
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B29">
         <v>5</v>
       </c>
       <c r="C29" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D29" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="E29" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="F29" t="s">
         <v>41</v>
       </c>
       <c r="G29" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="H29" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="I29" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="J29" t="s">
         <v>17</v>
@@ -1875,25 +1896,25 @@
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B30">
         <v>1</v>
       </c>
       <c r="C30" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="D30" t="s">
+        <v>180</v>
+      </c>
+      <c r="E30" t="s">
+        <v>181</v>
+      </c>
+      <c r="F30" t="s">
+        <v>41</v>
+      </c>
+      <c r="G30" t="s">
         <v>179</v>
-      </c>
-      <c r="E30" t="s">
-        <v>180</v>
-      </c>
-      <c r="F30" t="s">
-        <v>178</v>
-      </c>
-      <c r="G30" t="s">
-        <v>181</v>
       </c>
       <c r="H30" t="s">
         <v>182</v>
@@ -1905,8 +1926,40 @@
         <v>17</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
+        <v>184</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>185</v>
+      </c>
+      <c r="D31" t="s">
+        <v>186</v>
+      </c>
+      <c r="E31" t="s">
+        <v>187</v>
+      </c>
+      <c r="F31" t="s">
+        <v>185</v>
+      </c>
+      <c r="G31" t="s">
+        <v>188</v>
+      </c>
+      <c r="H31" t="s">
+        <v>189</v>
+      </c>
+      <c r="I31" t="s">
+        <v>190</v>
+      </c>
+      <c r="J31" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
         <v>41</v>
       </c>
     </row>

</xml_diff>

<commit_message>
corrected the RX TX connection of BLE
</commit_message>
<xml_diff>
--- a/PCB/BOM.xlsx
+++ b/PCB/BOM.xlsx
@@ -4,14 +4,14 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="BOM_Board1_PCB2_2026-04-13" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="BOM_Board1_1_PCB2_2_2026-05-12" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="202">
   <si>
     <t>No.</t>
   </si>
@@ -94,7 +94,7 @@
     <t>10uF</t>
   </si>
   <si>
-    <t>C14,C18</t>
+    <t>C14,C14.2,C18</t>
   </si>
   <si>
     <t>CL10A106MQ8NNNC</t>
@@ -202,7 +202,7 @@
     <t>KT-0603Y</t>
   </si>
   <si>
-    <t>LED1,LED2,LED3,LED4,LED5</t>
+    <t>LED1,LED2,LED3,LED4,LED5,LED6,LED7</t>
   </si>
   <si>
     <t>LED0603-R-RD</t>
@@ -283,10 +283,31 @@
     <t>14</t>
   </si>
   <si>
+    <t>1.4kΩ</t>
+  </si>
+  <si>
+    <t>R0,R31,R32,R33,R34,R35</t>
+  </si>
+  <si>
+    <t>R0402</t>
+  </si>
+  <si>
+    <t>0402WGF1401TCE</t>
+  </si>
+  <si>
+    <t>UNI-ROYAL(厚声)</t>
+  </si>
+  <si>
+    <t>C39650</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
     <t>1kΩ</t>
   </si>
   <si>
-    <t>R19,R21,R22</t>
+    <t>R19,R21,R21.2,R22</t>
   </si>
   <si>
     <t>R1206</t>
@@ -295,13 +316,10 @@
     <t>1206W4J0102T5E</t>
   </si>
   <si>
-    <t>UNI-ROYAL(厚声)</t>
-  </si>
-  <si>
     <t>C1469</t>
   </si>
   <si>
-    <t>15</t>
+    <t>16</t>
   </si>
   <si>
     <t>1MΩ</t>
@@ -316,7 +334,7 @@
     <t>C17927</t>
   </si>
   <si>
-    <t>16</t>
+    <t>17</t>
   </si>
   <si>
     <t>10kΩ</t>
@@ -334,7 +352,7 @@
     <t>C25612</t>
   </si>
   <si>
-    <t>17</t>
+    <t>18</t>
   </si>
   <si>
     <t>190pF@1kHz</t>
@@ -355,7 +373,7 @@
     <t>C8760</t>
   </si>
   <si>
-    <t>18</t>
+    <t>19</t>
   </si>
   <si>
     <t>47kΩ</t>
@@ -373,24 +391,6 @@
     <t>C620684</t>
   </si>
   <si>
-    <t>19</t>
-  </si>
-  <si>
-    <t>1.4kΩ</t>
-  </si>
-  <si>
-    <t>R31,R32,R33,R34,R35</t>
-  </si>
-  <si>
-    <t>R0402</t>
-  </si>
-  <si>
-    <t>0402WGF1401TCE</t>
-  </si>
-  <si>
-    <t>C39650</t>
-  </si>
-  <si>
     <t>20</t>
   </si>
   <si>
@@ -448,6 +448,21 @@
     <t>23</t>
   </si>
   <si>
+    <t>100kΩ</t>
+  </si>
+  <si>
+    <t>R49,R50,R51,R52,R53</t>
+  </si>
+  <si>
+    <t>0402WGF1003TCE</t>
+  </si>
+  <si>
+    <t>C25741</t>
+  </si>
+  <si>
+    <t>24</t>
+  </si>
+  <si>
     <t>4*4*1.7 贴片</t>
   </si>
   <si>
@@ -460,7 +475,7 @@
     <t>C10852</t>
   </si>
   <si>
-    <t>24</t>
+    <t>25</t>
   </si>
   <si>
     <t>EL817S1(B)(TU)-F</t>
@@ -478,7 +493,7 @@
     <t>C63268</t>
   </si>
   <si>
-    <t>25</t>
+    <t>26</t>
   </si>
   <si>
     <t>STM32F103C8T6</t>
@@ -493,7 +508,7 @@
     <t>C8734</t>
   </si>
   <si>
-    <t>26</t>
+    <t>27</t>
   </si>
   <si>
     <t>HLK-5M03</t>
@@ -511,7 +526,7 @@
     <t>C209906</t>
   </si>
   <si>
-    <t>27</t>
+    <t>28</t>
   </si>
   <si>
     <t>DS1021-1x2SF11-B</t>
@@ -529,7 +544,7 @@
     <t>C7430358</t>
   </si>
   <si>
-    <t>28</t>
+    <t>29</t>
   </si>
   <si>
     <t>MOC3053SM</t>
@@ -547,7 +562,7 @@
     <t>C899829</t>
   </si>
   <si>
-    <t>29</t>
+    <t>30</t>
   </si>
   <si>
     <t>AMS1117-3.3V</t>
@@ -565,7 +580,25 @@
     <t>C2688239</t>
   </si>
   <si>
-    <t>30</t>
+    <t>31</t>
+  </si>
+  <si>
+    <t>BLE-SER-A-ANT</t>
+  </si>
+  <si>
+    <t>U24</t>
+  </si>
+  <si>
+    <t>custom SMD</t>
+  </si>
+  <si>
+    <t>WCH(南京沁恒)</t>
+  </si>
+  <si>
+    <t>C2829462</t>
+  </si>
+  <si>
+    <t>32</t>
   </si>
   <si>
     <t>8MHz</t>
@@ -960,7 +993,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J32"/>
+  <dimension ref="A1:J34"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="10" width="20" customWidth="1"/>
@@ -1067,7 +1100,7 @@
         <v>25</v>
       </c>
       <c r="B4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C4" t="s">
         <v>26</v>
@@ -1259,7 +1292,7 @@
         <v>61</v>
       </c>
       <c r="B10">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C10" t="s">
         <v>62</v>
@@ -1419,7 +1452,7 @@
         <v>89</v>
       </c>
       <c r="B15">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C15" t="s">
         <v>90</v>
@@ -1451,7 +1484,7 @@
         <v>96</v>
       </c>
       <c r="B16">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C16" t="s">
         <v>97</v>
@@ -1460,19 +1493,19 @@
         <v>98</v>
       </c>
       <c r="E16" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="F16" t="s">
         <v>97</v>
       </c>
       <c r="G16" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="H16" t="s">
         <v>94</v>
       </c>
       <c r="I16" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J16" t="s">
         <v>17</v>
@@ -1480,22 +1513,22 @@
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B17">
         <v>1</v>
       </c>
       <c r="C17" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D17" t="s">
+        <v>104</v>
+      </c>
+      <c r="E17" t="s">
+        <v>99</v>
+      </c>
+      <c r="F17" t="s">
         <v>103</v>
-      </c>
-      <c r="E17" t="s">
-        <v>104</v>
-      </c>
-      <c r="F17" t="s">
-        <v>102</v>
       </c>
       <c r="G17" t="s">
         <v>105</v>
@@ -1533,10 +1566,10 @@
         <v>111</v>
       </c>
       <c r="H18" t="s">
+        <v>94</v>
+      </c>
+      <c r="I18" t="s">
         <v>112</v>
-      </c>
-      <c r="I18" t="s">
-        <v>113</v>
       </c>
       <c r="J18" t="s">
         <v>17</v>
@@ -1544,28 +1577,28 @@
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>113</v>
+      </c>
+      <c r="B19">
+        <v>1</v>
+      </c>
+      <c r="C19" t="s">
         <v>114</v>
       </c>
-      <c r="B19">
-        <v>2</v>
-      </c>
-      <c r="C19" t="s">
+      <c r="D19" t="s">
         <v>115</v>
       </c>
-      <c r="D19" t="s">
+      <c r="E19" t="s">
         <v>116</v>
       </c>
-      <c r="E19" t="s">
+      <c r="F19" t="s">
+        <v>114</v>
+      </c>
+      <c r="G19" t="s">
         <v>117</v>
       </c>
-      <c r="F19" t="s">
-        <v>115</v>
-      </c>
-      <c r="G19" t="s">
+      <c r="H19" t="s">
         <v>118</v>
-      </c>
-      <c r="H19" t="s">
-        <v>94</v>
       </c>
       <c r="I19" t="s">
         <v>119</v>
@@ -1579,7 +1612,7 @@
         <v>120</v>
       </c>
       <c r="B20">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C20" t="s">
         <v>121</v>
@@ -1620,7 +1653,7 @@
         <v>128</v>
       </c>
       <c r="E21" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="F21" t="s">
         <v>127</v>
@@ -1707,7 +1740,7 @@
         <v>144</v>
       </c>
       <c r="B24">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C24" t="s">
         <v>145</v>
@@ -1716,16 +1749,16 @@
         <v>146</v>
       </c>
       <c r="E24" t="s">
+        <v>92</v>
+      </c>
+      <c r="F24" t="s">
+        <v>145</v>
+      </c>
+      <c r="G24" t="s">
         <v>147</v>
       </c>
-      <c r="F24" t="s">
-        <v>41</v>
-      </c>
-      <c r="G24" t="s">
-        <v>145</v>
-      </c>
       <c r="H24" t="s">
-        <v>54</v>
+        <v>94</v>
       </c>
       <c r="I24" t="s">
         <v>148</v>
@@ -1757,10 +1790,10 @@
         <v>150</v>
       </c>
       <c r="H25" t="s">
+        <v>54</v>
+      </c>
+      <c r="I25" t="s">
         <v>153</v>
-      </c>
-      <c r="I25" t="s">
-        <v>154</v>
       </c>
       <c r="J25" t="s">
         <v>17</v>
@@ -1768,28 +1801,28 @@
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B26">
         <v>1</v>
       </c>
       <c r="C26" t="s">
+        <v>155</v>
+      </c>
+      <c r="D26" t="s">
         <v>156</v>
       </c>
-      <c r="D26" t="s">
+      <c r="E26" t="s">
         <v>157</v>
-      </c>
-      <c r="E26" t="s">
-        <v>158</v>
       </c>
       <c r="F26" t="s">
         <v>41</v>
       </c>
       <c r="G26" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="H26" t="s">
-        <v>87</v>
+        <v>158</v>
       </c>
       <c r="I26" t="s">
         <v>159</v>
@@ -1821,10 +1854,10 @@
         <v>161</v>
       </c>
       <c r="H27" t="s">
+        <v>87</v>
+      </c>
+      <c r="I27" t="s">
         <v>164</v>
-      </c>
-      <c r="I27" t="s">
-        <v>165</v>
       </c>
       <c r="J27" t="s">
         <v>17</v>
@@ -1832,31 +1865,31 @@
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
+        <v>165</v>
+      </c>
+      <c r="B28">
+        <v>1</v>
+      </c>
+      <c r="C28" t="s">
         <v>166</v>
       </c>
-      <c r="B28">
-        <v>4</v>
-      </c>
-      <c r="C28" t="s">
+      <c r="D28" t="s">
         <v>167</v>
       </c>
-      <c r="D28" t="s">
+      <c r="E28" t="s">
         <v>168</v>
-      </c>
-      <c r="E28" t="s">
-        <v>169</v>
       </c>
       <c r="F28" t="s">
         <v>41</v>
       </c>
       <c r="G28" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H28" t="s">
+        <v>169</v>
+      </c>
+      <c r="I28" t="s">
         <v>170</v>
-      </c>
-      <c r="I28" t="s">
-        <v>171</v>
       </c>
       <c r="J28" t="s">
         <v>17</v>
@@ -1864,31 +1897,31 @@
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
+        <v>171</v>
+      </c>
+      <c r="B29">
+        <v>4</v>
+      </c>
+      <c r="C29" t="s">
         <v>172</v>
       </c>
-      <c r="B29">
-        <v>5</v>
-      </c>
-      <c r="C29" t="s">
+      <c r="D29" t="s">
         <v>173</v>
       </c>
-      <c r="D29" t="s">
+      <c r="E29" t="s">
         <v>174</v>
-      </c>
-      <c r="E29" t="s">
-        <v>175</v>
       </c>
       <c r="F29" t="s">
         <v>41</v>
       </c>
       <c r="G29" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="H29" t="s">
+        <v>175</v>
+      </c>
+      <c r="I29" t="s">
         <v>176</v>
-      </c>
-      <c r="I29" t="s">
-        <v>177</v>
       </c>
       <c r="J29" t="s">
         <v>17</v>
@@ -1896,31 +1929,31 @@
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
+        <v>177</v>
+      </c>
+      <c r="B30">
+        <v>5</v>
+      </c>
+      <c r="C30" t="s">
         <v>178</v>
       </c>
-      <c r="B30">
-        <v>1</v>
-      </c>
-      <c r="C30" t="s">
+      <c r="D30" t="s">
         <v>179</v>
       </c>
-      <c r="D30" t="s">
+      <c r="E30" t="s">
         <v>180</v>
-      </c>
-      <c r="E30" t="s">
-        <v>181</v>
       </c>
       <c r="F30" t="s">
         <v>41</v>
       </c>
       <c r="G30" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="H30" t="s">
+        <v>181</v>
+      </c>
+      <c r="I30" t="s">
         <v>182</v>
-      </c>
-      <c r="I30" t="s">
-        <v>183</v>
       </c>
       <c r="J30" t="s">
         <v>17</v>
@@ -1928,38 +1961,102 @@
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B31">
         <v>1</v>
       </c>
       <c r="C31" t="s">
+        <v>184</v>
+      </c>
+      <c r="D31" t="s">
         <v>185</v>
       </c>
-      <c r="D31" t="s">
+      <c r="E31" t="s">
         <v>186</v>
       </c>
-      <c r="E31" t="s">
+      <c r="F31" t="s">
+        <v>41</v>
+      </c>
+      <c r="G31" t="s">
+        <v>184</v>
+      </c>
+      <c r="H31" t="s">
         <v>187</v>
       </c>
-      <c r="F31" t="s">
-        <v>185</v>
-      </c>
-      <c r="G31" t="s">
+      <c r="I31" t="s">
         <v>188</v>
       </c>
-      <c r="H31" t="s">
+      <c r="J31" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
         <v>189</v>
       </c>
-      <c r="I31" t="s">
+      <c r="B32">
+        <v>1</v>
+      </c>
+      <c r="C32" t="s">
         <v>190</v>
       </c>
-      <c r="J31" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
+      <c r="D32" t="s">
+        <v>191</v>
+      </c>
+      <c r="E32" t="s">
+        <v>192</v>
+      </c>
+      <c r="F32" t="s">
+        <v>41</v>
+      </c>
+      <c r="G32" t="s">
+        <v>190</v>
+      </c>
+      <c r="H32" t="s">
+        <v>193</v>
+      </c>
+      <c r="I32" t="s">
+        <v>194</v>
+      </c>
+      <c r="J32" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>195</v>
+      </c>
+      <c r="B33">
+        <v>1</v>
+      </c>
+      <c r="C33" t="s">
+        <v>196</v>
+      </c>
+      <c r="D33" t="s">
+        <v>197</v>
+      </c>
+      <c r="E33" t="s">
+        <v>198</v>
+      </c>
+      <c r="F33" t="s">
+        <v>196</v>
+      </c>
+      <c r="G33" t="s">
+        <v>199</v>
+      </c>
+      <c r="H33" t="s">
+        <v>200</v>
+      </c>
+      <c r="I33" t="s">
+        <v>201</v>
+      </c>
+      <c r="J33" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
         <v>41</v>
       </c>
     </row>

</xml_diff>